<commit_message>
Charge the Challenge's Lab4 hours to week 9 AC
The leads put 6 h of Lab4 (workflow, alerts and ADR) above their level
of effort in week 9. They now count in AC (+120 USD, covered by the
contingency: 1,344 to 1,224 USD) while EV stays the same, since Lab4 is
not in the baseline. CPI goes from 1.03 to 1.01; SPI stays at 1.03.
Same change in the Steering 2 workbook and the steering page.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/Steering 2.xlsx
+++ b/outputs/Steering 2.xlsx
@@ -6576,7 +6576,7 @@
     <row r="27">
       <c r="K27" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Leads como level of effort: su trabajo no se cierra por paquetes, así que EV = PV. AC: 18 h reales/sem de devs + 16 h reales/sem de leads + lo facturado de infra e IA. El detalle está en la hoja Avance semanal.</t>
+          <t xml:space="preserve">• Leads como level of effort: su trabajo no se cierra por paquetes, así que EV = PV. AC: 18 h reales/sem de devs + 16 h reales/sem de leads (22 h en la semana 9 por el challenge) + lo facturado de infra e IA. El detalle está en la hoja Avance semanal.</t>
         </is>
       </c>
     </row>
@@ -6618,7 +6618,7 @@
     <row r="33">
       <c r="K33" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Divisor de 227,62 h: las 225,62 h del Cronograma v4 (78 paquetes, con la épica 13.0 sumada el 07/10) con 13.1 re-estimada de 4 h a 6 h (Lab2: SPO-276 y SPO-277, ADR-001). Lab4 (workflow, alertas y ADR, 6 h) lo hicieron los leads y queda dentro de su level of effort.</t>
+          <t xml:space="preserve">• Divisor de 227,62 h: las 225,62 h del Cronograma v4 (78 paquetes, con la épica 13.0 sumada el 07/10) con 13.1 re-estimada de 4 h a 6 h (Lab2: SPO-276 y SPO-277, ADR-001). Lab4 (workflow, alertas y ADR, 6 h) lo hicieron los leads por encima de su level of effort: suma 6 h × 20 USD = 120 USD al AC de la semana 9 y se cubre con la contingencia (1.344 → 1.224 USD). El EV no cambia porque Lab4 no está en la línea base.</t>
         </is>
       </c>
     </row>
@@ -7198,11 +7198,11 @@
         <f>(PRESUPUESTO!J15+PRESUPUESTO!J16+PRESUPUESTO!J17+PRESUPUESTO!J18)/'Curva S'!$L$22</f>
       </c>
       <c r="M14" s="47">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="N14" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cierran 5.1.1, 5.1.4, 6.4.3, 7.1.3, 7.3.1, 11.1.2, 11.2.2, 13.1.1, 13.1.2 (challenge, 13.1 re-estimada a 6 h)</t>
+          <t xml:space="preserve">Cierran 5.1.1, 5.1.4, 6.4.3, 7.1.3, 7.3.1, 11.1.2, 11.2.2, 13.1.1, 13.1.2 (challenge, 13.1 re-estimada a 6 h) · Leads: +6 h de Lab4 (workflow, alertas y ADR), de la contingencia</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
     <row r="21">
       <c r="A21" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Horas plan y reales (devs): 3 devs × 6 h/sem, de las filas de devs de PRESUPUESTO; reales 18 h/sem. Horas leads: 4 leads × 4 h/sem, de las filas 15 a 18 de PRESUPUESTO; reales 16 h/sem.</t>
+          <t xml:space="preserve">• Horas plan y reales (devs): 3 devs × 6 h/sem, de las filas de devs de PRESUPUESTO; reales 18 h/sem. Horas leads: 4 leads × 4 h/sem, de las filas 15 a 18 de PRESUPUESTO; reales 16 h/sem (22 h en la semana 9: +6 h de Lab4 por el challenge, cubiertas con la contingencia).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Steering 2: activity contingency (10 %) inside the BAC and the EVM
- steering.html v2: PV and EV x1.1 (contingencyInEvm), BAC 7.391,36;
  management contingency (10 %) shown as reserve outside the BAC, total
  budget 8.063,30. Steering 1 keeps what was presented.
- Steering 2.xlsx: Curva S!L7 = 10 % parameter, PRESUPUESTO row 19 with
  the weekly contingency, EV formula x(1 + L7), notes updated. Edited in
  the XML so charts and styles stay intact; recalculated in Excel.
- Tests: v2 expectations updated (the old ones predated the Lab4 hours).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/Steering 2.xlsx
+++ b/outputs/Steering 2.xlsx
@@ -502,7 +502,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
@@ -625,6 +625,9 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="20" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="15" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -4372,20 +4375,51 @@
         <f t="shared" si="0"/>
       </c>
     </row>
-    <row r="19" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B19" s="50"/>
-      <c r="C19" s="50"/>
-      <c r="D19" s="50"/>
-      <c r="E19" s="50"/>
-      <c r="F19" s="50"/>
-      <c r="G19" s="50"/>
-      <c r="H19" s="50"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="50"/>
-      <c r="K19" s="50"/>
-      <c r="L19" s="50"/>
-      <c r="M19" s="50"/>
-      <c r="N19" s="50"/>
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contingencia de actividades · 10 % del costo de la semana (Curva S!L7, dentro del BAC)</t>
+        </is>
+      </c>
+      <c r="B19" s="50">
+        <f>'Curva S'!$L$7*SUM(B9:B18)</f>
+      </c>
+      <c r="C19" s="50">
+        <f>'Curva S'!$L$7*SUM(C9:C18)</f>
+      </c>
+      <c r="D19" s="50">
+        <f>'Curva S'!$L$7*SUM(D9:D18)</f>
+      </c>
+      <c r="E19" s="50">
+        <f>'Curva S'!$L$7*SUM(E9:E18)</f>
+      </c>
+      <c r="F19" s="50">
+        <f>'Curva S'!$L$7*SUM(F9:F18)</f>
+      </c>
+      <c r="G19" s="50">
+        <f>'Curva S'!$L$7*SUM(G9:G18)</f>
+      </c>
+      <c r="H19" s="50">
+        <f>'Curva S'!$L$7*SUM(H9:H18)</f>
+      </c>
+      <c r="I19" s="50">
+        <f>'Curva S'!$L$7*SUM(I9:I18)</f>
+      </c>
+      <c r="J19" s="50">
+        <f>'Curva S'!$L$7*SUM(J9:J18)</f>
+      </c>
+      <c r="K19" s="50">
+        <f>'Curva S'!$L$7*SUM(K9:K18)</f>
+      </c>
+      <c r="L19" s="50">
+        <f>'Curva S'!$L$7*SUM(L9:L18)</f>
+      </c>
+      <c r="M19" s="50">
+        <f>'Curva S'!$L$7*SUM(M9:M18)</f>
+      </c>
+      <c r="N19" s="50">
+        <f>'Curva S'!$L$7*SUM(N9:N18)</f>
+      </c>
       <c r="O19" s="50"/>
       <c r="P19" s="50"/>
       <c r="Q19" s="50"/>
@@ -5854,7 +5888,7 @@
     <row r="2">
       <c r="A2" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Equipo 11 · Corte 15/10/2026 (semana 10, cierre del S2) · USD acumulados (devs + leads + infra + IA) · Base: WBS y Cronograma v4 · Datos desde PRESUPUESTO y Avance semanal</t>
+          <t xml:space="preserve">Equipo 11 · Corte 15/10/2026 (semana 10, cierre del S2) · USD acumulados (devs + leads + infra + IA + 10 % de contingencia de actividades) · Base: WBS y Cronograma v4 · Datos desde PRESUPUESTO y Avance semanal</t>
         </is>
       </c>
     </row>
@@ -6027,11 +6061,11 @@
       </c>
       <c r="K7" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">BAC total del proyecto (USD)</t>
-        </is>
-      </c>
-      <c r="L7" s="31">
-        <v>8063.3</v>
+          <t xml:space="preserve">Contingencia de actividades (% del costo, dentro del BAC)</t>
+        </is>
+      </c>
+      <c r="L7" s="54">
+        <v>0.1</v>
       </c>
     </row>
     <row r="8">
@@ -6068,7 +6102,7 @@
       </c>
       <c r="K8" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">BAC línea base EVM (devs + leads + infra + IA)</t>
+          <t xml:space="preserve">BAC línea base EVM = BAC del proyecto (devs + leads + infra + IA + contingencia de actividades)</t>
         </is>
       </c>
       <c r="L8" s="38">
@@ -6555,7 +6589,7 @@
     <row r="24">
       <c r="K24" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• PV: 3 devs (6 h/sem × 10 USD/h = 60 USD/sem c/u) + 4 leads (PM, PO, Tech Lead y QA Lead: 4 h/sem × 20 USD/h = 80 USD/sem c/u) durante 13 semanas + Azure B1 desde el deploy (29/08) + Claude Code/ChatGPT (3 × 20 USD/mes). La semana de reserva (05/11 → 12/11) es reserva de gestión y no entra.</t>
+          <t xml:space="preserve">• PV: 3 devs (6 h/sem × 10 USD/h = 60 USD/sem c/u) + 4 leads (PM, PO, Tech Lead y QA Lead: 4 h/sem × 20 USD/h = 80 USD/sem c/u) durante 13 semanas + Azure B1 desde el deploy (29/08) + Claude Code/ChatGPT (3 × 20 USD/mes). No entran la reserva de gestión (contingencia de gestión, 10 % = 671,94 USD) ni la semana de reserva (05/11 → 12/11).</t>
         </is>
       </c>
     </row>
@@ -6569,7 +6603,7 @@
     <row r="26">
       <c r="K26" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• EV = EV desarrollo + EV leads. EV desarrollo = % completo × BAC desarrollo (L21); % completo = horas estimadas de los paquetes de la WBS cerrados / 227,62 h. Semanal: 5,5 · 32,71 · 8,72 · 30,3 · 26,29 · 20,18 · 7,83 · 21,14 · 24,42 · 16,22 h (193,31 h).</t>
+          <t xml:space="preserve">• EV = (EV desarrollo + EV leads) × (1 + contingencia de actividades). EV desarrollo = % completo × BAC desarrollo (L21); % completo = horas estimadas de los paquetes de la WBS cerrados / 227,62 h. Semanal: 5,5 · 32,71 · 8,72 · 30,3 · 26,29 · 20,18 · 7,83 · 21,14 · 24,42 · 16,22 h (193,31 h).</t>
         </is>
       </c>
     </row>
@@ -6583,7 +6617,7 @@
     <row r="28">
       <c r="K28" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• EAC, ETC y VAC usan el BAC de la línea base EVM (L8), la misma base que PV, EV y AC. BAC total del proyecto: 442 HH + infra e IA + 20 % de contingencia = 8.063,30 USD, sin CAPEX.</t>
+          <t xml:space="preserve">• Contingencia en el EVM (cambio respecto del Steering 1): la contingencia de actividades (10 %) es parte de la línea base de costos (PMBOK 7.3), así que se reparte en proporción al trabajo planificado (fila 19 de PRESUPUESTO) y PV y EV van × 1,1. El BAC del EVM (L8) es el BAC del proyecto: 6.719,42 + 10 % = 7.391,36 USD, sin CAPEX. La contingencia de gestión (otro 10 %, 671,94 USD) es reserva de gestión: queda fuera del BAC y del EVM. Presupuesto total: 8.063,30 USD. El AC es el gasto real, también el que cubre la contingencia. El CPI incluye la contingencia no usada: sin ella da 1,01.</t>
         </is>
       </c>
     </row>
@@ -6618,7 +6652,7 @@
     <row r="33">
       <c r="K33" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Divisor de 227,62 h: las 225,62 h del Cronograma v4 (78 paquetes, con la épica 13.0 sumada el 07/10) con 13.1 re-estimada de 4 h a 6 h (Lab2: SPO-276 y SPO-277, ADR-001). Lab4 (workflow, alertas y ADR, 6 h) lo hicieron los leads por encima de su level of effort: suma 6 h × 20 USD = 120 USD al AC de la semana 9 y se cubre con la contingencia (1.344 → 1.224 USD). El EV no cambia porque Lab4 no está en la línea base.</t>
+          <t xml:space="preserve">• Divisor de 227,62 h: las 225,62 h del Cronograma v4 (78 paquetes, con la épica 13.0 sumada el 07/10) con 13.1 re-estimada de 4 h a 6 h (Lab2: SPO-276 y SPO-277, ADR-001). Lab4 (workflow, alertas y ADR, 6 h) lo hicieron los leads por encima de su level of effort: suma 6 h × 20 USD = 120 USD al AC de la semana 9 y se cubre con la contingencia de actividades (671,94 → 551,94 USD). El EV no cambia porque Lab4 no está en la línea base.</t>
         </is>
       </c>
     </row>
@@ -6732,7 +6766,7 @@
       </c>
       <c r="J5" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">EV total (USD) = % × BAC desarrollo + leads</t>
+          <t xml:space="preserve">EV total (USD) = (% × BAC desarrollo + leads) × (1 + contingencia de actividades)</t>
         </is>
       </c>
       <c r="K5" s="25" t="inlineStr">
@@ -6789,7 +6823,7 @@
         <f>H6</f>
       </c>
       <c r="J6" s="45">
-        <f>G6*'Curva S'!$L$21+L6*'Curva S'!$L$22</f>
+        <f>(G6*'Curva S'!$L$21+L6*'Curva S'!$L$22)*(1+'Curva S'!$L$7)</f>
       </c>
       <c r="K6" s="45">
         <f>E6*'Curva S'!$L$6+I6+M6*'Curva S'!$L$22</f>
@@ -6839,7 +6873,7 @@
         <f>H7</f>
       </c>
       <c r="J7" s="45">
-        <f>G7*'Curva S'!$L$21+L7*'Curva S'!$L$22</f>
+        <f>(G7*'Curva S'!$L$21+L7*'Curva S'!$L$22)*(1+'Curva S'!$L$7)</f>
       </c>
       <c r="K7" s="45">
         <f>E7*'Curva S'!$L$6+I7+M7*'Curva S'!$L$22</f>
@@ -6889,7 +6923,7 @@
         <f>H8</f>
       </c>
       <c r="J8" s="45">
-        <f>G8*'Curva S'!$L$21+L8*'Curva S'!$L$22</f>
+        <f>(G8*'Curva S'!$L$21+L8*'Curva S'!$L$22)*(1+'Curva S'!$L$7)</f>
       </c>
       <c r="K8" s="45">
         <f>E8*'Curva S'!$L$6+I8+M8*'Curva S'!$L$22</f>
@@ -6939,7 +6973,7 @@
         <f>H9</f>
       </c>
       <c r="J9" s="45">
-        <f>G9*'Curva S'!$L$21+L9*'Curva S'!$L$22</f>
+        <f>(G9*'Curva S'!$L$21+L9*'Curva S'!$L$22)*(1+'Curva S'!$L$7)</f>
       </c>
       <c r="K9" s="45">
         <f>E9*'Curva S'!$L$6+I9+M9*'Curva S'!$L$22</f>
@@ -6989,7 +7023,7 @@
         <f>H10</f>
       </c>
       <c r="J10" s="45">
-        <f>G10*'Curva S'!$L$21+L10*'Curva S'!$L$22</f>
+        <f>(G10*'Curva S'!$L$21+L10*'Curva S'!$L$22)*(1+'Curva S'!$L$7)</f>
       </c>
       <c r="K10" s="45">
         <f>E10*'Curva S'!$L$6+I10+M10*'Curva S'!$L$22</f>
@@ -7039,7 +7073,7 @@
         <f>H11</f>
       </c>
       <c r="J11" s="45">
-        <f>G11*'Curva S'!$L$21+L11*'Curva S'!$L$22</f>
+        <f>(G11*'Curva S'!$L$21+L11*'Curva S'!$L$22)*(1+'Curva S'!$L$7)</f>
       </c>
       <c r="K11" s="45">
         <f>E11*'Curva S'!$L$6+I11+M11*'Curva S'!$L$22</f>
@@ -7089,7 +7123,7 @@
         <f>H12</f>
       </c>
       <c r="J12" s="45">
-        <f>G12*'Curva S'!$L$21+L12*'Curva S'!$L$22</f>
+        <f>(G12*'Curva S'!$L$21+L12*'Curva S'!$L$22)*(1+'Curva S'!$L$7)</f>
       </c>
       <c r="K12" s="45">
         <f>E12*'Curva S'!$L$6+I12+M12*'Curva S'!$L$22</f>
@@ -7139,7 +7173,7 @@
         <f>H13</f>
       </c>
       <c r="J13" s="45">
-        <f>G13*'Curva S'!$L$21+L13*'Curva S'!$L$22</f>
+        <f>(G13*'Curva S'!$L$21+L13*'Curva S'!$L$22)*(1+'Curva S'!$L$7)</f>
       </c>
       <c r="K13" s="45">
         <f>E13*'Curva S'!$L$6+I13+M13*'Curva S'!$L$22</f>
@@ -7189,7 +7223,7 @@
         <f>H14</f>
       </c>
       <c r="J14" s="45">
-        <f>G14*'Curva S'!$L$21+L14*'Curva S'!$L$22</f>
+        <f>(G14*'Curva S'!$L$21+L14*'Curva S'!$L$22)*(1+'Curva S'!$L$7)</f>
       </c>
       <c r="K14" s="45">
         <f>E14*'Curva S'!$L$6+I14+M14*'Curva S'!$L$22</f>
@@ -7239,7 +7273,7 @@
         <f>H15</f>
       </c>
       <c r="J15" s="46">
-        <f>G15*'Curva S'!$L$21+L15*'Curva S'!$L$22</f>
+        <f>(G15*'Curva S'!$L$21+L15*'Curva S'!$L$22)*(1+'Curva S'!$L$7)</f>
       </c>
       <c r="K15" s="46">
         <f>E15*'Curva S'!$L$6+I15+M15*'Curva S'!$L$22</f>
@@ -7439,7 +7473,7 @@
     <row r="24">
       <c r="A24" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• EV total = % completo × BAC desarrollo (Curva S!L21) + horas leads plan × tarifa leads (level of effort: EV = PV). AC total = horas reales devs × tarifa dev + horas reales leads × tarifa leads + Infra/IA facturados. Ambas columnas alimentan las filas 41 y 43 de PRESUPUESTO.</t>
+          <t xml:space="preserve">• EV total = (% completo × BAC desarrollo (Curva S!L21) + horas leads plan × tarifa leads) × (1 + contingencia de actividades, Curva S!L7). Leads como level of effort: EV = PV. AC total = horas reales devs × tarifa dev + horas reales leads × tarifa leads + Infra/IA facturados (sin contingencia: es gasto real). Ambas columnas alimentan las filas 41 y 43 de PRESUPUESTO.</t>
         </is>
       </c>
     </row>

</xml_diff>